<commit_message>
Ingest ASIA full 5-year statements (2564-2568)
Added ASIA Q1-Q3 + FY for all five years via ingest.py (20 statements from
nested zips). ASIA now complete 5x4; overall coverage 56 quarterly rows.

Validation: 432 checks, 0 errors. One expected warning — ASIA Q4/2564 gross
margin -8.4% — verified as real COVID-trough data (FY2564 whole-year GM
-0.6%, net loss 211M), not an extraction fault: Q1+Q2+Q3+Q4 reconcile to FY
and the balance check passes. The 5-year path is a clean recovery (net loss
211M->3M, DSO 95->23 days).

Regenerated TOUR_all_linked.xlsx, ASIA_quarterly_linked.xlsx, metrics_all.csv,
ratios_report.xlsx with ASIA filled across all five years.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjBjdz26s52MeASaozo8gq
</commit_message>
<xml_diff>
--- a/tour-finance/output/ASIA_quarterly_linked.xlsx
+++ b/tour-finance/output/ASIA_quarterly_linked.xlsx
@@ -48,12 +48,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -598,38 +598,70 @@
           <t>รายได้รวม</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="4">
+      <c r="B2" t="n">
+        <v>161.421</v>
+      </c>
+      <c r="C2" t="n">
+        <v>143.655</v>
+      </c>
+      <c r="D2" t="n">
+        <v>146.768</v>
+      </c>
+      <c r="E2" s="3">
         <f>F2-B2-C2-D2</f>
         <v/>
       </c>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="4">
+      <c r="F2" t="n">
+        <v>599.845</v>
+      </c>
+      <c r="G2" t="n">
+        <v>173.164</v>
+      </c>
+      <c r="H2" t="n">
+        <v>210.576</v>
+      </c>
+      <c r="I2" t="n">
+        <v>255.119</v>
+      </c>
+      <c r="J2" s="3">
         <f>K2-G2-H2-I2</f>
         <v/>
       </c>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="4">
+      <c r="K2" t="n">
+        <v>924.299</v>
+      </c>
+      <c r="L2" t="n">
+        <v>299.966</v>
+      </c>
+      <c r="M2" t="n">
+        <v>289.335</v>
+      </c>
+      <c r="N2" t="n">
+        <v>307.831</v>
+      </c>
+      <c r="O2" s="3">
         <f>P2-L2-M2-N2</f>
         <v/>
       </c>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="4">
+      <c r="P2" t="n">
+        <v>1188.482</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>316.06</v>
+      </c>
+      <c r="R2" t="n">
+        <v>306.951</v>
+      </c>
+      <c r="S2" t="n">
+        <v>326.359</v>
+      </c>
+      <c r="T2" s="3">
         <f>U2-Q2-R2-S2</f>
         <v/>
       </c>
-      <c r="U2" s="3" t="n"/>
+      <c r="U2" t="n">
+        <v>1275.109</v>
+      </c>
       <c r="V2" t="n">
         <v>342.684</v>
       </c>
@@ -639,7 +671,7 @@
       <c r="X2" t="n">
         <v>321.648</v>
       </c>
-      <c r="Y2" s="4">
+      <c r="Y2" s="3">
         <f>Z2-V2-W2-X2</f>
         <v/>
       </c>
@@ -653,38 +685,70 @@
           <t>รายได้อื่น</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="4">
+      <c r="B3" t="n">
+        <v>12.568</v>
+      </c>
+      <c r="C3" t="n">
+        <v>13.539</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8.788</v>
+      </c>
+      <c r="E3" s="3">
         <f>F3-B3-C3-D3</f>
         <v/>
       </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="4">
+      <c r="F3" t="n">
+        <v>48.375</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10.123</v>
+      </c>
+      <c r="H3" t="n">
+        <v>11.369</v>
+      </c>
+      <c r="I3" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="J3" s="3">
         <f>K3-G3-H3-I3</f>
         <v/>
       </c>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="4">
+      <c r="K3" t="n">
+        <v>45.181</v>
+      </c>
+      <c r="L3" t="n">
+        <v>15.717</v>
+      </c>
+      <c r="M3" t="n">
+        <v>16.357</v>
+      </c>
+      <c r="N3" t="n">
+        <v>22.347</v>
+      </c>
+      <c r="O3" s="3">
         <f>P3-L3-M3-N3</f>
         <v/>
       </c>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="4">
+      <c r="P3" t="n">
+        <v>72.435</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>15.012</v>
+      </c>
+      <c r="R3" t="n">
+        <v>19.732</v>
+      </c>
+      <c r="S3" t="n">
+        <v>15.012</v>
+      </c>
+      <c r="T3" s="3">
         <f>U3-Q3-R3-S3</f>
         <v/>
       </c>
-      <c r="U3" s="3" t="n"/>
+      <c r="U3" t="n">
+        <v>77.119</v>
+      </c>
       <c r="V3" t="n">
         <v>19.762</v>
       </c>
@@ -694,7 +758,7 @@
       <c r="X3" t="n">
         <v>23.877</v>
       </c>
-      <c r="Y3" s="4">
+      <c r="Y3" s="3">
         <f>Z3-V3-W3-X3</f>
         <v/>
       </c>
@@ -708,38 +772,70 @@
           <t>ต้นทุนขาย (จริง)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="4">
+      <c r="B4" t="n">
+        <v>155.453</v>
+      </c>
+      <c r="C4" t="n">
+        <v>150.548</v>
+      </c>
+      <c r="D4" t="n">
+        <v>137.157</v>
+      </c>
+      <c r="E4" s="3">
         <f>F4-B4-C4-D4</f>
         <v/>
       </c>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="4">
+      <c r="F4" t="n">
+        <v>603.606</v>
+      </c>
+      <c r="G4" t="n">
+        <v>161.775</v>
+      </c>
+      <c r="H4" t="n">
+        <v>179.281</v>
+      </c>
+      <c r="I4" t="n">
+        <v>201.105</v>
+      </c>
+      <c r="J4" s="3">
         <f>K4-G4-H4-I4</f>
         <v/>
       </c>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="4">
+      <c r="K4" t="n">
+        <v>747.973</v>
+      </c>
+      <c r="L4" t="n">
+        <v>219.817</v>
+      </c>
+      <c r="M4" t="n">
+        <v>220.397</v>
+      </c>
+      <c r="N4" t="n">
+        <v>223.495</v>
+      </c>
+      <c r="O4" s="3">
         <f>P4-L4-M4-N4</f>
         <v/>
       </c>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="4">
+      <c r="P4" t="n">
+        <v>876.527</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>220.309</v>
+      </c>
+      <c r="R4" t="n">
+        <v>222.275</v>
+      </c>
+      <c r="S4" t="n">
+        <v>241.647</v>
+      </c>
+      <c r="T4" s="3">
         <f>U4-Q4-R4-S4</f>
         <v/>
       </c>
-      <c r="U4" s="3" t="n"/>
+      <c r="U4" t="n">
+        <v>921.247</v>
+      </c>
       <c r="V4" t="n">
         <v>233.19</v>
       </c>
@@ -749,7 +845,7 @@
       <c r="X4" t="n">
         <v>236.609</v>
       </c>
-      <c r="Y4" s="4">
+      <c r="Y4" s="3">
         <f>Z4-V4-W4-X4</f>
         <v/>
       </c>
@@ -763,38 +859,70 @@
           <t>กำไรสุทธิ (รวม)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="4">
+      <c r="B5" t="n">
+        <v>-48.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-58.89</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-37.553</v>
+      </c>
+      <c r="E5" s="3">
         <f>F5-B5-C5-D5</f>
         <v/>
       </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="4">
+      <c r="F5" t="n">
+        <v>-210.623</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-49.978</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-35.144</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-25.28</v>
+      </c>
+      <c r="J5" s="3">
         <f>K5-G5-H5-I5</f>
         <v/>
       </c>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="4">
+      <c r="K5" t="n">
+        <v>-112.271</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-13.24</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-5.875</v>
+      </c>
+      <c r="N5" t="n">
+        <v>5.997</v>
+      </c>
+      <c r="O5" s="3">
         <f>P5-L5-M5-N5</f>
         <v/>
       </c>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3" t="n"/>
-      <c r="T5" s="4">
+      <c r="P5" t="n">
+        <v>-60.57</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-4.117</v>
+      </c>
+      <c r="S5" t="n">
+        <v>-4.096</v>
+      </c>
+      <c r="T5" s="3">
         <f>U5-Q5-R5-S5</f>
         <v/>
       </c>
-      <c r="U5" s="3" t="n"/>
+      <c r="U5" t="n">
+        <v>-5.596</v>
+      </c>
       <c r="V5" t="n">
         <v>14.423</v>
       </c>
@@ -804,7 +932,7 @@
       <c r="X5" t="n">
         <v>-6.092</v>
       </c>
-      <c r="Y5" s="4">
+      <c r="Y5" s="3">
         <f>Z5-V5-W5-X5</f>
         <v/>
       </c>
@@ -818,50 +946,66 @@
           <t>กำไรสุทธิ (ส่วนแม่)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="4">
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" t="n">
+        <v>-58.854</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-36.74</v>
+      </c>
+      <c r="E6" s="3">
         <f>F6-B6-C6-D6</f>
         <v/>
       </c>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="4">
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" t="n">
+        <v>-35.074</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-24.879</v>
+      </c>
+      <c r="J6" s="3">
         <f>K6-G6-H6-I6</f>
         <v/>
       </c>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="4">
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" t="n">
+        <v>-5.349</v>
+      </c>
+      <c r="N6" t="n">
+        <v>6.344</v>
+      </c>
+      <c r="O6" s="3">
         <f>P6-L6-M6-N6</f>
         <v/>
       </c>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="4">
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" t="n">
+        <v>-3.459</v>
+      </c>
+      <c r="S6" t="n">
+        <v>-3.001</v>
+      </c>
+      <c r="T6" s="3">
         <f>U6-Q6-R6-S6</f>
         <v/>
       </c>
-      <c r="U6" s="3" t="n"/>
-      <c r="V6" s="3" t="n"/>
+      <c r="U6" s="4" t="n"/>
+      <c r="V6" s="4" t="n"/>
       <c r="W6" t="n">
         <v>-14.469</v>
       </c>
       <c r="X6" t="n">
         <v>-5.466</v>
       </c>
-      <c r="Y6" s="4">
+      <c r="Y6" s="3">
         <f>Z6-V6-W6-X6</f>
         <v/>
       </c>
-      <c r="Z6" s="3" t="n"/>
+      <c r="Z6" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -998,22 +1142,54 @@
           <t>ลูกหนี้การค้า</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
+      <c r="B2" t="n">
+        <v>136.25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>145.444</v>
+      </c>
+      <c r="D2" t="n">
+        <v>139.641</v>
+      </c>
+      <c r="E2" t="n">
+        <v>198.409</v>
+      </c>
+      <c r="F2" t="n">
+        <v>134.447</v>
+      </c>
+      <c r="G2" t="n">
+        <v>140.663</v>
+      </c>
+      <c r="H2" t="n">
+        <v>142.238</v>
+      </c>
+      <c r="I2" t="n">
+        <v>127.504</v>
+      </c>
+      <c r="J2" t="n">
+        <v>137.68</v>
+      </c>
+      <c r="K2" t="n">
+        <v>150.621</v>
+      </c>
+      <c r="L2" t="n">
+        <v>143.885</v>
+      </c>
+      <c r="M2" t="n">
+        <v>149.662</v>
+      </c>
+      <c r="N2" t="n">
+        <v>122.044</v>
+      </c>
+      <c r="O2" t="n">
+        <v>125.417</v>
+      </c>
+      <c r="P2" t="n">
+        <v>115.971</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>105.384</v>
+      </c>
       <c r="R2" t="n">
         <v>87.279</v>
       </c>
@@ -1036,22 +1212,54 @@
           <t>สินค้าคงเหลือ</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
+      <c r="B3" t="n">
+        <v>40.331</v>
+      </c>
+      <c r="C3" t="n">
+        <v>39.374</v>
+      </c>
+      <c r="D3" t="n">
+        <v>39.459</v>
+      </c>
+      <c r="E3" t="n">
+        <v>39.702</v>
+      </c>
+      <c r="F3" t="n">
+        <v>39.693</v>
+      </c>
+      <c r="G3" t="n">
+        <v>39.429</v>
+      </c>
+      <c r="H3" t="n">
+        <v>39.954</v>
+      </c>
+      <c r="I3" t="n">
+        <v>39.43</v>
+      </c>
+      <c r="J3" t="n">
+        <v>40.001</v>
+      </c>
+      <c r="K3" t="n">
+        <v>40.924</v>
+      </c>
+      <c r="L3" t="n">
+        <v>41.095</v>
+      </c>
+      <c r="M3" t="n">
+        <v>42.135</v>
+      </c>
+      <c r="N3" t="n">
+        <v>43.539</v>
+      </c>
+      <c r="O3" t="n">
+        <v>43.141</v>
+      </c>
+      <c r="P3" t="n">
+        <v>43.78</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>44.865</v>
+      </c>
       <c r="R3" t="n">
         <v>46.247</v>
       </c>
@@ -1074,22 +1282,54 @@
           <t>เจ้าหนี้การค้า</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
+      <c r="B4" t="n">
+        <v>21.655</v>
+      </c>
+      <c r="C4" t="n">
+        <v>17.226</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13.107</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18.514</v>
+      </c>
+      <c r="F4" t="n">
+        <v>14.131</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16.515</v>
+      </c>
+      <c r="H4" t="n">
+        <v>21.681</v>
+      </c>
+      <c r="I4" t="n">
+        <v>24.026</v>
+      </c>
+      <c r="J4" t="n">
+        <v>24.926</v>
+      </c>
+      <c r="K4" t="n">
+        <v>27.178</v>
+      </c>
+      <c r="L4" t="n">
+        <v>24.927</v>
+      </c>
+      <c r="M4" t="n">
+        <v>27.801</v>
+      </c>
+      <c r="N4" t="n">
+        <v>27.136</v>
+      </c>
+      <c r="O4" t="n">
+        <v>29.724</v>
+      </c>
+      <c r="P4" t="n">
+        <v>28.136</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>34.269</v>
+      </c>
       <c r="R4" t="n">
         <v>33.155</v>
       </c>
@@ -1112,22 +1352,54 @@
           <t>สินทรัพย์รวม</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3" t="n"/>
+      <c r="B5" t="n">
+        <v>9569.273999999999</v>
+      </c>
+      <c r="C5" t="n">
+        <v>9453.575999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9433.053</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9416.727000000001</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10500.936</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10401.72</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10389.057</v>
+      </c>
+      <c r="I5" t="n">
+        <v>10415.012</v>
+      </c>
+      <c r="J5" t="n">
+        <v>10456.552</v>
+      </c>
+      <c r="K5" t="n">
+        <v>10324.99</v>
+      </c>
+      <c r="L5" t="n">
+        <v>10277.756</v>
+      </c>
+      <c r="M5" t="n">
+        <v>10250.041</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10212.295</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10195.015</v>
+      </c>
+      <c r="P5" t="n">
+        <v>10337.145</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>10147.093</v>
+      </c>
       <c r="R5" t="n">
         <v>10140.751</v>
       </c>
@@ -1150,22 +1422,54 @@
           <t>ส่วนของเจ้าของรวม</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3" t="n"/>
+      <c r="B6" t="n">
+        <v>5340.39</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5272.208</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5225.804</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5220.527</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6070.568</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6056.51</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6057.951</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6077.899</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6092.038</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6072.954</v>
+      </c>
+      <c r="L6" t="n">
+        <v>6068.102</v>
+      </c>
+      <c r="M6" t="n">
+        <v>6085.32</v>
+      </c>
+      <c r="N6" t="n">
+        <v>6049.842</v>
+      </c>
+      <c r="O6" t="n">
+        <v>6075.806</v>
+      </c>
+      <c r="P6" t="n">
+        <v>6073.584</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>5982.58</v>
+      </c>
       <c r="R6" t="n">
         <v>6008.757</v>
       </c>
@@ -1188,22 +1492,54 @@
           <t>หนี้สินรวม</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3" t="n"/>
+      <c r="B7" t="n">
+        <v>4228.883</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4181.369</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4207.248</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4196.199</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4430.368</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4345.21</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4331.106</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4337.113</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4364.514</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4252.036</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4209.654</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4164.722</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4162.454</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4119.209</v>
+      </c>
+      <c r="P7" t="n">
+        <v>4263.561</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>4164.514</v>
+      </c>
       <c r="R7" t="n">
         <v>4131.994</v>
       </c>
@@ -2455,7 +2791,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ไตรมาสที่มีข้อมูลจริงแล้ว: Q1/2568, Q2/2568, Q3/2568, FY/2568</t>
+          <t>ไตรมาสที่มีข้อมูลจริงแล้ว: Q1/2564, Q2/2564, Q3/2564, FY/2564, Q1/2565, Q2/2565, Q3/2565, FY/2565, Q1/2566, Q2/2566, Q3/2566, FY/2566, Q1/2567, Q2/2567, Q3/2567, FY/2567, Q1/2568, Q2/2568, Q3/2568, FY/2568</t>
         </is>
       </c>
     </row>

</xml_diff>